<commit_message>
S152 5절: 마감 - 1,701건 3분 28초 · 케이스 160/160 · 감사 넷 불변 (미해결 70 -> 80)
착수 3분 50초 · 마감 3분 28초 (1번 PC · 둘 다 깨끗한 판 · 22초 차는 안 갈랐다).
케이스 도구 134.5초 · 회귀값 여덟 불변 · 기상 취득 0회.
감사 957·807·961·808 불변 · ruff check pass · mypy 10건/파일 둘 · scan_ctrl 0곳.
src·tests·tools·data diff 빈 출력. 「다음 작업」 칸은 S150 판치를 걷어 2,897자.
OPEN_ITEMS 갈래 넷에 열을 이름으로 세웠다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LEPxreDkEvdHdB85AHz9BH
</commit_message>
<xml_diff>
--- a/output/casestudy_20260908.xlsx
+++ b/output/casestudy_20260908.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>10.7458086000006</v>
+        <v>11.9448521000013</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>11.46569060000184</v>
+        <v>11.65679319999981</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>7.855843400000595</v>
+        <v>7.518661999998585</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>12.09897619999902</v>
+        <v>12.33852979999938</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>11.86837970000124</v>
+        <v>13.07490949999919</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>10.97934379999788</v>
+        <v>11.22078159999728</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>13.63354229999823</v>
+        <v>13.60031639999943</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>14.16431209999791</v>
+        <v>12.14657689999876</v>
       </c>
     </row>
     <row r="10">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>17.9200353999986</v>
+        <v>17.85023329999967</v>
       </c>
     </row>
     <row r="11">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>9.084609000001365</v>
+        <v>8.027737500000512</v>
       </c>
     </row>
     <row r="12">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>7.661419600000954</v>
+        <v>6.643039999999019</v>
       </c>
     </row>
   </sheetData>
@@ -13998,7 +13998,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10.7 초</t>
+          <t>11.9 초</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14010,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11.5 초</t>
+          <t>11.7 초</t>
         </is>
       </c>
     </row>
@@ -14022,7 +14022,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7.9 초</t>
+          <t>7.5 초</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12.1 초</t>
+          <t>12.3 초</t>
         </is>
       </c>
     </row>
@@ -14046,7 +14046,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>11.9 초</t>
+          <t>13.1 초</t>
         </is>
       </c>
     </row>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.0 초</t>
+          <t>11.2 초</t>
         </is>
       </c>
     </row>
@@ -14082,7 +14082,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.2 초</t>
+          <t>12.1 초</t>
         </is>
       </c>
     </row>
@@ -14106,7 +14106,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9.1 초</t>
+          <t>8.0 초</t>
         </is>
       </c>
     </row>
@@ -14118,7 +14118,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7.7 초</t>
+          <t>6.6 초</t>
         </is>
       </c>
     </row>
@@ -14130,7 +14130,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>136.4 초</t>
+          <t>134.5 초</t>
         </is>
       </c>
     </row>

</xml_diff>